<commit_message>
📅 日报更新 2026-08-22 03:04
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-08-22.xlsx
+++ b/data/exports/黄老师/dist_order_2026-08-22.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>49493414</v>
+        <v>49508265</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>49493126</v>
+        <v>49493414</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>49492499</v>
+        <v>49493126</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>刘盼昭</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-21 22:44:53</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>49455301</v>
+        <v>49492499</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>红霞</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-21 22:29:43</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>49432023</v>
+        <v>49455301</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>周开平</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-20 22:46:59</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -425,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>49415939</v>
+        <v>49432023</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>花生米</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-20 11:55:45</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -464,17 +464,17 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
@@ -485,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>49415918</v>
+        <v>49415939</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>杨梅芳</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-19 22:48:58</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -545,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>49415913</v>
+        <v>49415918</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>心语无言</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-19 22:48:24</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -605,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>49415890</v>
+        <v>49415913</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>安好</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-19 22:48:18</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -660,21 +660,16 @@
       <c r="L10" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N10" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>49415874</v>
+        <v>49415890</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>雨夜聆风</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -699,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-19 22:47:56</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -725,16 +720,21 @@
       <c r="L11" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N11" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>49415871</v>
+        <v>49415874</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>飘</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-19 22:47:40</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -790,59 +790,119 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H13" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K13" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L13" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="0">
         <v>49415867</v>
       </c>
-      <c r="B13" s="0" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C13" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D13" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E13" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G13" s="0" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H13" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I13" s="0" t="inlineStr">
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
         <is>
           <t>黄老师-抖音01</t>
         </is>
       </c>
-      <c r="J13" s="0" t="inlineStr">
+      <c r="J14" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K13" s="0" t="inlineStr">
+      <c r="K14" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L13" s="0" t="inlineStr">
+      <c r="L14" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>